<commit_message>
email phone, website copy and edit option added
</commit_message>
<xml_diff>
--- a/excel/Batch_01_Leads_Tracker.xlsx
+++ b/excel/Batch_01_Leads_Tracker.xlsx
@@ -34,7 +34,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="200" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -657,7 +657,7 @@
         <v>Landline: 0208 629 1723; Mobile: 07443 773 773</v>
       </c>
       <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">WhatsApp: https://wa.me/447443773773
+        <v xml:space="preserve">[x] WhatsApp: https://wa.me/447443773773
 Checkatrade: https://www.checkatrade.com/trades/yourchoicelocksandglazing
 Contact page: https://yourchoicelocksmiths.co.uk/your_choice_locksmiths_service_contact_us</v>
       </c>

</xml_diff>